<commit_message>
Limite de 1 camisa por pessoa (por WhatsApp)
- Servidor soma as camisas do WhatsApp em reservas não canceladas
- Limite vem da aba Configurações (Camisas por pessoa) e o site usa o valor do servidor
- Textos do site atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/bloco22-reservas.xlsx
+++ b/planilha/bloco22-reservas.xlsx
@@ -2180,13 +2180,17 @@
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="37" t="inlineStr">
         <is>
-          <t>Máximo de camisas por reserva</t>
+          <t>Camisas por pessoa (por WhatsApp)</t>
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>Soma todas as reservas não canceladas do mesmo WhatsApp.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="37" t="inlineStr">

</xml_diff>